<commit_message>
Template di importazione precompilati con i dati demo di pixora/demo-alina
- genera_demo_alina.py legge anagrafiche, budget e dipendenti dai moduli demo
  (senza eseguirli) e produce demo_alina/DEMO_ALINA_*.xlsx
- ID esterni dei moduli demo: il reimport aggiorna invece di duplicare
- Budget analitico con colonne per nome piano (Proprieta/Categoria/Natura)
- Esempi generici allineati ai codici del piano dei conti l10n_it

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013waGJG7pYcG8W9mHUJy7ny
</commit_message>
<xml_diff>
--- a/import_templates/04_Piano_dei_Conti.xlsx
+++ b/import_templates/04_Piano_dei_Conti.xlsx
@@ -207,7 +207,7 @@
       <text>
         <t>ID esterno
 [Consigliato]
-Formato: CONTO_6105
+Formato: CONTO_4214
 Per AGGIORNARE conti già esistenti (es. quelli di l10n_it) esportarli prima con "Compatibile con importazione" e usare l'ID esportato.</t>
       </text>
     </comment>
@@ -215,7 +215,7 @@
       <text>
         <t>Codice
 [OBBLIGATORIO]
-Formato: 6105
+Formato: 4214
 Univoco per azienda. Solo cifre/lettere/punti. Formattare la colonna come TESTO.</t>
       </text>
     </comment>
@@ -646,12 +646,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CONTO_6105</t>
+          <t>CONTO_4214</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>6105</t>
+          <t>4214</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -726,12 +726,12 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CONTO_4105</t>
+          <t>CONTO_3120</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>4105</t>
+          <t>3120</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>CONTO_6105</t>
+          <t>CONTO_4214</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>6105</t>
+          <t>4214</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">

</xml_diff>